<commit_message>
Final fixes: mapping column, README setup, contribution and AI-use statements
</commit_message>
<xml_diff>
--- a/docs/feature_harmonization_matrix.xlsx
+++ b/docs/feature_harmonization_matrix.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -1915,7 +1915,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -4034,7 +4034,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Pending: instructor extract and field mapping not provided</t>
+          <t>Not applicable: no instructor extract supplied; mapped directly from ARMD Dryad version 403223</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">

</xml_diff>